<commit_message>
Add Returns & Waterfall tab: Year-1 SPV payout (40%x85%x14M), gross-revenue 50/15 waterfall
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ntjkuUSmwseQSpKGRDLJU
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-07-17-capital-deployment-monthly.xlsx
+++ b/cinderella/Outputs/2026-07-17-capital-deployment-monthly.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment + Revenue" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns &amp; Waterfall" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,10 +17,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0;(#,##0);&quot;–&quot;"/>
+    <numFmt numFmtId="165" formatCode="0.00&quot;x&quot;"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,8 +63,30 @@
       <color rgb="00404040"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00000000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="001F6E5E"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -119,6 +143,11 @@
         <fgColor rgb="00808080"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BF9000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -132,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -170,6 +199,21 @@
     <xf numFmtId="0" fontId="2" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="12" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="12" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2803,4 +2847,440 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>Cinderella Corp — Returns &amp; Waterfall (one SPV, base case)  ·  seed 50%→1x, 15%→2x, then 15% pro-rata (GROSS revenue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="30" t="inlineStr">
+        <is>
+          <t>Base team revenue (gross / season)</t>
+        </is>
+      </c>
+      <c r="B3" s="32" t="n">
+        <v>14000000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="30" t="inlineStr">
+        <is>
+          <t>SPV team-revenue share</t>
+        </is>
+      </c>
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>85%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>SPV profit (breaks even before team rev)</t>
+        </is>
+      </c>
+      <c r="B5" s="32" t="n">
+        <v>11900000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="30" t="inlineStr">
+        <is>
+          <t>Parent ownership of SPV</t>
+        </is>
+      </c>
+      <c r="B6" s="33" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="30" t="inlineStr">
+        <is>
+          <t>→ Parent SPV distribution / yr (40%×85%×14M)</t>
+        </is>
+      </c>
+      <c r="B7" s="32" t="n">
+        <v>4760000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="30" t="inlineStr">
+        <is>
+          <t>Franchise fee (one-time, 2027)</t>
+        </is>
+      </c>
+      <c r="B8" s="32" t="n">
+        <v>1500000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="30" t="inlineStr">
+        <is>
+          <t>Mgmt fee /yr (2%×$15M)</t>
+        </is>
+      </c>
+      <c r="B9" s="32" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>Seed investment / 1x</t>
+        </is>
+      </c>
+      <c r="B10" s="32" t="n">
+        <v>1500000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>($)</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>2027</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>2028</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>2029</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>2030</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>2031</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>2032</v>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>PARENT GROSS REVENUE</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="n"/>
+      <c r="C13" s="18" t="n"/>
+      <c r="D13" s="18" t="n"/>
+      <c r="E13" s="18" t="n"/>
+      <c r="F13" s="18" t="n"/>
+      <c r="G13" s="18" t="n"/>
+      <c r="H13" s="18" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Franchise fee (one-time)</t>
+        </is>
+      </c>
+      <c r="B14" s="35" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="C14" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="36" t="n">
+        <v>1500000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Management fee (2%)</t>
+        </is>
+      </c>
+      <c r="B15" s="35" t="n">
+        <v>150000</v>
+      </c>
+      <c r="C15" s="35" t="n">
+        <v>300000</v>
+      </c>
+      <c r="D15" s="35" t="n">
+        <v>300000</v>
+      </c>
+      <c r="E15" s="35" t="n">
+        <v>300000</v>
+      </c>
+      <c r="F15" s="35" t="n">
+        <v>300000</v>
+      </c>
+      <c r="G15" s="35" t="n">
+        <v>300000</v>
+      </c>
+      <c r="H15" s="36" t="n">
+        <v>1650000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SPV distribution (40% of profit)</t>
+        </is>
+      </c>
+      <c r="B16" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="35" t="n">
+        <v>4760000</v>
+      </c>
+      <c r="D16" s="35" t="n">
+        <v>4760000</v>
+      </c>
+      <c r="E16" s="35" t="n">
+        <v>4760000</v>
+      </c>
+      <c r="F16" s="35" t="n">
+        <v>4760000</v>
+      </c>
+      <c r="G16" s="35" t="n">
+        <v>4760000</v>
+      </c>
+      <c r="H16" s="36" t="n">
+        <v>23800000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  TOTAL parent gross revenue</t>
+        </is>
+      </c>
+      <c r="B17" s="38" t="n">
+        <v>1650000</v>
+      </c>
+      <c r="C17" s="38" t="n">
+        <v>5060000</v>
+      </c>
+      <c r="D17" s="38" t="n">
+        <v>5060000</v>
+      </c>
+      <c r="E17" s="38" t="n">
+        <v>5060000</v>
+      </c>
+      <c r="F17" s="38" t="n">
+        <v>5060000</v>
+      </c>
+      <c r="G17" s="38" t="n">
+        <v>5060000</v>
+      </c>
+      <c r="H17" s="38" t="n">
+        <v>26950000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="39" t="inlineStr">
+        <is>
+          <t>WATERFALL — to seed investors</t>
+        </is>
+      </c>
+      <c r="B18" s="40" t="n"/>
+      <c r="C18" s="40" t="n"/>
+      <c r="D18" s="40" t="n"/>
+      <c r="E18" s="40" t="n"/>
+      <c r="F18" s="40" t="n"/>
+      <c r="G18" s="40" t="n"/>
+      <c r="H18" s="40" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  To SEED investors (50/15/pro-rata)</t>
+        </is>
+      </c>
+      <c r="B19" s="42" t="n">
+        <v>825000</v>
+      </c>
+      <c r="C19" s="42" t="n">
+        <v>1231500</v>
+      </c>
+      <c r="D19" s="42" t="n">
+        <v>759000</v>
+      </c>
+      <c r="E19" s="42" t="n">
+        <v>759000</v>
+      </c>
+      <c r="F19" s="42" t="n">
+        <v>759000</v>
+      </c>
+      <c r="G19" s="42" t="n">
+        <v>759000</v>
+      </c>
+      <c r="H19" s="42" t="n">
+        <v>5092500</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Seed cumulative received</t>
+        </is>
+      </c>
+      <c r="B20" s="35" t="n">
+        <v>825000</v>
+      </c>
+      <c r="C20" s="35" t="n">
+        <v>2056500</v>
+      </c>
+      <c r="D20" s="35" t="n">
+        <v>2815500</v>
+      </c>
+      <c r="E20" s="35" t="n">
+        <v>3574500</v>
+      </c>
+      <c r="F20" s="35" t="n">
+        <v>4333500</v>
+      </c>
+      <c r="G20" s="35" t="n">
+        <v>5092500</v>
+      </c>
+      <c r="H20" s="36" t="n">
+        <v>18697500</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Seed MOIC</t>
+        </is>
+      </c>
+      <c r="B21" s="44" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="C21" s="44" t="n">
+        <v>1.371</v>
+      </c>
+      <c r="D21" s="44" t="n">
+        <v>1.877</v>
+      </c>
+      <c r="E21" s="44" t="n">
+        <v>2.383</v>
+      </c>
+      <c r="F21" s="44" t="n">
+        <v>2.889</v>
+      </c>
+      <c r="G21" s="44" t="n">
+        <v>3.395</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  To parent / common (retained)</t>
+        </is>
+      </c>
+      <c r="B22" s="35" t="n">
+        <v>825000</v>
+      </c>
+      <c r="C22" s="35" t="n">
+        <v>3828500</v>
+      </c>
+      <c r="D22" s="35" t="n">
+        <v>4301000</v>
+      </c>
+      <c r="E22" s="35" t="n">
+        <v>4301000</v>
+      </c>
+      <c r="F22" s="35" t="n">
+        <v>4301000</v>
+      </c>
+      <c r="G22" s="35" t="n">
+        <v>4301000</v>
+      </c>
+      <c r="H22" s="36" t="n">
+        <v>21857500</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="45" t="inlineStr">
+        <is>
+          <t>Return of capital (1×) reached: 2028   ·   2× reached: 2030   ·   ~3.4× by 2032 + residual equity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="30" t="inlineStr">
+        <is>
+          <t>Year-1 SPV payout: SPV breaks even before team revenue, so profit = team-rev share = $14.0M × 85% = $11.9M. Parent's 40% = $4.76M, paid end of SPV Year 1 (2028).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="30" t="inlineStr">
+        <is>
+          <t>Waterfall runs on parent GROSS revenue (per your instruction): 50¢/$1 to seed until 1× ($1.5M), then 15¢/$1 until 2× ($3.0M), then 15% pro-rata (regular payouts).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
+          <t>One SPV / one team, base case, team revenue held flat across the 5 SPV seasons (2027-28 → 2031-32; distributions 2028-2032). Additional cohorts multiply this — the franchise curve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="30" t="inlineStr">
+        <is>
+          <t>Seed is largely returned within ~2 years of the raise; 2× by 2030; residual equity beyond. Franchise + mgmt fees are the parent's early money, the 40% distribution is the back-end.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A27:H27"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>